<commit_message>
BP : nouvelle cap table 50/25/25 (sortie de Nazeh, parts → Nessim + Lamine)
Nazeh sort entièrement ; le BP passe de 40/25/25/10 à 50/25/25.
Chiffres recalculés (vérifiés par 3 chemins : site, simulateur live, xlsx) :
- Nessim : 3,56 M → 4,36 M DT (4 355 179) | multiple 11,9× → 14,5× | TRI ~82 % → ~90 %
- Ali / Lamine : 2,00 M chacun (inchangés)
- Net cumulé 11,9 M / total distribué 8,35 M / trésorerie min +278 k : inchangés
- Pre-money apports industrie : ~450 k → ~300 k (2 associés au lieu de 3)

Fichiers : index.html (cap table, pie chart, cartes, équipe), simulateur.html
(SH + arrays + chart 3 barres), BP_HCTECH_2025_RevenueShare.md, ONE_PAGER.md,
README.md, NOTE_INNOVATION_STARTUP_ACT.md, NOTE_APPROCHE_SICAR.md,
model/build_model.py + dividends.py, BP_HCTECH_7ans.xlsx régénéré.
Les (40 %) restants = part station (revenue share 60/40), volontairement intacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BP_HCTECH_7ans.xlsx
+++ b/BP_HCTECH_7ans.xlsx
@@ -715,7 +715,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>82 %</t>
+          <t>90 %</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>3,556,144 DT</t>
+          <t>4,355,179 DT</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>300000</v>
@@ -2522,17 +2522,17 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Nazeh Ben Ammar</t>
+          <t>Ali Ben Hamoud</t>
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>0.1</v>
+        <v>0.25</v>
       </c>
       <c r="C7" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>75000</v>
+        <v>150000</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Ali Ben Hamoud</t>
+          <t>Lamine</t>
         </is>
       </c>
       <c r="B8" s="21" t="n">
@@ -2553,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>187500</v>
+        <v>150000</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -2562,126 +2562,92 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Lamine</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>187500</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>Apport industrie/nature (techno, réseau, gestion)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B9" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="24" t="n">
+      <c r="C9" s="24" t="n">
         <v>300000</v>
       </c>
-      <c r="D10" s="24" t="n">
-        <v>750000</v>
-      </c>
-      <c r="E10" s="22" t="inlineStr"/>
+      <c r="D9" s="24" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E9" s="22" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Note : Nessim finance 100 % du capital (300 k) pour 50 %. Les parts d'Ali et Lamine</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Note : Nessim finance 100 % du capital (300 k) pour 40 %. Les parts des autres associés</t>
+          <t>correspondent à des apports en industrie/nature (exclusivité GEKO, réseau pétrolier, gestion)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>correspondent à des apports en industrie/nature (exclusivité GEKO, réseau pétrolier, gestion)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>valorisés ~450 k DT pre-money. À formaliser dans le pacte d'actionnaires.</t>
+          <t>valorisés ~300 k DT pre-money. À formaliser dans le pacte d'actionnaires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>Dividendes reçus sur 7 ans (Option 1) :</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
-        <is>
-          <t>Dividendes reçus sur 7 ans (Option 1) :</t>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Nessim Mami</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" s="26" t="n">
+        <v>4355179.397675838</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>14.5× le capital</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nessim Mami</t>
+          <t>Ali Ben Hamoud</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" s="26" t="n">
-        <v>3556143.518140671</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>11.9× le capital</t>
-        </is>
-      </c>
+        <v>1997589.698837919</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Nazeh Ben Ammar</t>
+          <t>Lamine</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" s="26" t="n">
-        <v>799035.8795351677</v>
+        <v>1997589.698837919</v>
       </c>
       <c r="E18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Ali Ben Hamoud</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" s="26" t="n">
-        <v>1997589.698837919</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Lamine</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" s="26" t="n">
-        <v>1997589.698837919</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2698,7 +2664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2722,7 +2688,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nessim encaisse 100% jusqu'à capital + prime 20% (360k), puis pro-rata 40/10/25/25 · payout 70%</t>
+          <t>Nessim encaisse 100% jusqu'à capital + prime 20% (360k), puis pro-rata 50/25/25 · payout 70%</t>
         </is>
       </c>
     </row>
@@ -2787,32 +2753,32 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>Nessim Mami (40 %)</t>
+          <t>Nessim Mami (50 %)</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
         <v>93431.89439165924</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>312730.514476095</v>
+        <v>324271.1166930336</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>281553.7558319576</v>
+        <v>351942.194789947</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>428205.6075370688</v>
+        <v>535257.009421336</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>606441.0940194725</v>
+        <v>758051.3675243405</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>806610.3186033876</v>
+        <v>1008262.898254234</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>1027170.33328103</v>
+        <v>1283962.916601288</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>3556143.518140671</v>
+        <v>4355179.397675838</v>
       </c>
     </row>
     <row r="7">
@@ -2878,76 +2844,45 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Nazeh Ben Ammar (10 %)</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>11540.60221693856</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <v>70388.43895798939</v>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>107051.4018842672</v>
-      </c>
-      <c r="F9" s="11" t="n">
-        <v>151610.2735048681</v>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>201652.5796508469</v>
-      </c>
-      <c r="H9" s="11" t="n">
-        <v>256792.5833202575</v>
-      </c>
-      <c r="I9" s="11" t="n">
-        <v>799035.8795351677</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>TOTAL distribué</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B9" s="18" t="n">
         <v>93431.89439165924</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C9" s="18" t="n">
         <v>381974.1277777264</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D9" s="18" t="n">
         <v>703884.3895798939</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E9" s="18" t="n">
         <v>1070514.018842672</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F9" s="18" t="n">
         <v>1516102.735048681</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G9" s="18" t="n">
         <v>2016525.796508469</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H9" s="18" t="n">
         <v>2567925.833202575</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I9" s="18" t="n">
         <v>8350358.795351677</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Nessim : capital remboursé fin An 2 · TRI ≈ 90 % · multiple 14.5× · total reçu 4,355,179 DT</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>Nessim : capital remboursé fin An 2 · TRI ≈ 82 % · multiple 11.9× · total reçu 3,556,144 DT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Note : dividende déclaré au titre de l'exercice N, versé en N+1. 30 % du résultat conservé en réserve.</t>
         </is>

</xml_diff>

<commit_message>
Dossier leasing : tableur Excel à formules + mini-site, abandon SICAR
- HCTECH_BP_Leasing.xlsx (+ model/build_bp_leasing.py) : classeur à formules
  vivantes, 12 onglets. États financiers prévisionnels normés (État de résultat,
  Bilan équilibré, Flux de trésorerie), Ratios financiers (EBITDA, marges, DSCR,
  ROE), Capacité leasing, Dividendes. Vérifié par recalcul (moteur formulas).
- leasing.html : mini-site de présentation pour les sociétés de leasing
  (lien à partager) — pitch, chiffres, couverture, téléchargement du dossier.
- Abandon SICAR : NOTE_APPROCHE_SICAR.md supprimé (modèle leasing = pas de levée).
- Rappel : BP déjà passé en leasing 5 ans + cap table 45/25/25/5, Nazeh = conseiller.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BP_HCTECH_7ans.xlsx
+++ b/BP_HCTECH_7ans.xlsx
@@ -583,7 +583,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>3,668,465 DT</t>
+          <t>3,738,417 DT</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>11,929,084 DT</t>
+          <t>10,990,449 DT</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>13,655,709 DT</t>
+          <t>12,744,278 DT</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>19,468 DT</t>
+          <t>16,276 DT</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>12,271 DT</t>
+          <t>15,463 DT</t>
         </is>
       </c>
     </row>
@@ -715,7 +715,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>90 %</t>
+          <t>78 %</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>4,355,179 DT</t>
+          <t>3,659,992 DT</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>8,350,359 DT</t>
+          <t>7,693,315 DT</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>7,873,276 DT</t>
+          <t>7,667,855 DT</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>1022.578679102493</v>
+        <v>1288.565243267147</v>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
@@ -1798,25 +1798,25 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>-200425.4211040887</v>
+        <v>-252558.7876803608</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>-544011.8572825266</v>
+        <v>-685516.7094181221</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>-887598.2934609643</v>
+        <v>-1118474.631155883</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>-1231184.729639402</v>
+        <v>-1551432.552893645</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>-1574771.16581784</v>
+        <v>-1984390.474631406</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>-1918357.601996278</v>
+        <v>-2164789.608688807</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>-2261944.038174715</v>
+        <v>-2164789.608688807</v>
       </c>
     </row>
     <row r="9">
@@ -1938,25 +1938,25 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>185380.7428405938</v>
+        <v>133247.3762643218</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>757885.1741621555</v>
+        <v>616380.32202656</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1396596.011071218</v>
+        <v>1165719.673376299</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>2124035.751671968</v>
+        <v>1803787.928417725</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>3008140.347318812</v>
+        <v>2598521.038505245</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>4001043.247040614</v>
+        <v>3754611.240348085</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>5095090.938894</v>
+        <v>5192245.368379908</v>
       </c>
     </row>
     <row r="14">
@@ -1966,25 +1966,25 @@
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>-51906.60799536626</v>
+        <v>-37309.26535401009</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>-212207.8487654036</v>
+        <v>-172586.4901674368</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>-391046.8830999411</v>
+        <v>-326401.5085453637</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>-594730.0104681511</v>
+        <v>-505060.6199569632</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>-842279.2972492673</v>
+        <v>-727585.8907814688</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>-1120292.109171372</v>
+        <v>-1051291.147297464</v>
       </c>
       <c r="H14" s="11" t="n">
-        <v>-1426625.46289032</v>
+        <v>-1453828.703146374</v>
       </c>
     </row>
     <row r="15">
@@ -1994,25 +1994,25 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>133474.1348452275</v>
+        <v>95938.11091031166</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>545677.325396752</v>
+        <v>443793.8318591232</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>1005549.127971277</v>
+        <v>839318.1648309352</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>1529305.741203817</v>
+        <v>1298727.308460762</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>2165861.050069544</v>
+        <v>1870935.147723777</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>2880751.137869242</v>
+        <v>2703320.093050621</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>3668465.476003679</v>
+        <v>3738416.665233533</v>
       </c>
     </row>
     <row r="16">
@@ -2022,25 +2022,25 @@
         </is>
       </c>
       <c r="B16" s="18" t="n">
-        <v>133474.1348452275</v>
+        <v>95938.11091031166</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>679151.4602419795</v>
+        <v>539731.9427694349</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>1684700.588213257</v>
+        <v>1379050.10760037</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>3214006.329417074</v>
+        <v>2677777.416061132</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>5379867.379486619</v>
+        <v>4548712.563784909</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>8260618.51735586</v>
+        <v>7252032.65683553</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>11929083.99335954</v>
+        <v>10990449.32206906</v>
       </c>
     </row>
   </sheetData>
@@ -2144,25 +2144,25 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>133474.1348452275</v>
+        <v>95938.11091031166</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>545677.325396752</v>
+        <v>443793.8318591232</v>
       </c>
       <c r="D6" s="11" t="n">
-        <v>1005549.127971277</v>
+        <v>839318.1648309352</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1529305.741203817</v>
+        <v>1298727.308460762</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>2165861.050069544</v>
+        <v>1870935.147723777</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>2880751.137869242</v>
+        <v>2703320.093050621</v>
       </c>
       <c r="H6" s="11" t="n">
-        <v>3668465.476003679</v>
+        <v>3738416.665233533</v>
       </c>
     </row>
     <row r="7">
@@ -2172,25 +2172,25 @@
         </is>
       </c>
       <c r="B7" s="11" t="n">
-        <v>485380.7428405938</v>
+        <v>433247.3762643219</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>1191359.309007383</v>
+        <v>1012318.432936872</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>2375747.471313197</v>
+        <v>2005451.616145733</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>4108736.339885224</v>
+        <v>3482838.036018096</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>6522146.676735889</v>
+        <v>5576298.45456638</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>9680910.62652724</v>
+        <v>8603323.804132998</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>13655709.45624987</v>
+        <v>12744278.02521544</v>
       </c>
     </row>
     <row r="8">
@@ -2203,22 +2203,22 @@
         <v>0</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>93431.89439165918</v>
+        <v>67156.67763721815</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>475406.0221693856</v>
+        <v>377812.3599386043</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>1179290.41174928</v>
+        <v>965335.0753202587</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>2249804.430591952</v>
+        <v>1874444.191242792</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>3765907.165640633</v>
+        <v>3184098.794649436</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>5782432.962149101</v>
+        <v>5076422.859784871</v>
       </c>
     </row>
     <row r="9">
@@ -2228,25 +2228,25 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>485380.7428405938</v>
+        <v>433247.3762643219</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>1097927.414615724</v>
+        <v>945161.755299654</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>1900341.449143811</v>
+        <v>1627639.256207129</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>2929445.928135945</v>
+        <v>2517502.960697837</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>4272342.246143937</v>
+        <v>3701854.263323588</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>5915003.460886608</v>
+        <v>5419225.009483562</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>7873276.494100771</v>
+        <v>7667855.165430572</v>
       </c>
     </row>
     <row r="11">
@@ -2387,12 +2387,12 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>-12,271 DT/an</t>
+          <t>-15,463 DT/an</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>57 928 @ 12 %/7 ans</t>
+          <t>57 928 @ 12 %/5 ans (pdt 5 ans, puis 0)</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       </c>
       <c r="B12" s="20" t="inlineStr">
         <is>
-          <t>19,468 DT/an</t>
+          <t>16,276 DT/an</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -2440,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="B6" s="21" t="n">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="C6" s="11" t="n">
         <v>300000</v>
@@ -2532,7 +2532,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>150000</v>
+        <v>166666.6666666667</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -2553,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>150000</v>
+        <v>166666.6666666667</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -2562,92 +2562,126 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Nazeh Ben Ammar</t>
+        </is>
+      </c>
+      <c r="B9" s="21" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>33333.33333333334</v>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Apport industrie/nature (techno, réseau, gestion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B10" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C10" s="24" t="n">
         <v>300000</v>
       </c>
-      <c r="D9" s="24" t="n">
-        <v>600000</v>
-      </c>
-      <c r="E9" s="22" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Note : Nessim finance 100 % du capital (300 k) pour 50 %. Les parts d'Ali et Lamine</t>
-        </is>
-      </c>
+      <c r="D10" s="24" t="n">
+        <v>666666.6666666666</v>
+      </c>
+      <c r="E10" s="22" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>correspondent à des apports en industrie/nature (exclusivité GEKO, réseau pétrolier, gestion)</t>
+          <t>Note : Nessim finance 100 % du capital (300 k) pour 45 %. Les parts d'Ali, Lamine et Nazeh</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>valorisés ~300 k DT pre-money. À formaliser dans le pacte d'actionnaires.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="25" t="inlineStr">
+          <t>correspondent à des apports en industrie/nature (exclusivité GEKO, réseau pétrolier, réseau institutionnel, gestion)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>valorisés ~367 k DT pre-money. À formaliser dans le pacte d'actionnaires.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>Dividendes reçus sur 7 ans (Option 1) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Nessim Mami</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" s="26" t="n">
-        <v>4355179.397675838</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>14.5× le capital</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ali Ben Hamoud</t>
+          <t>Nessim Mami</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr"/>
       <c r="D17" s="26" t="n">
-        <v>1997589.698837919</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>3659991.536451755</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>12.2× le capital</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lamine</t>
+          <t>Ali Ben Hamoud</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr"/>
       <c r="D18" s="26" t="n">
-        <v>1997589.698837919</v>
+        <v>1833328.631362086</v>
       </c>
       <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lamine</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" s="26" t="n">
+        <v>1833328.631362086</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Nazeh Ben Ammar</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" s="26" t="n">
+        <v>366665.7262724172</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2664,7 +2698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2688,7 +2722,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Nessim encaisse 100% jusqu'à capital + prime 20% (360k), puis pro-rata 50/25/25 · payout 70%</t>
+          <t>Nessim encaisse 100% jusqu'à capital + prime 20% (360k), puis pro-rata 45/25/25/5 · payout 70%</t>
         </is>
       </c>
     </row>
@@ -2753,32 +2787,32 @@
     <row r="6">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>Nessim Mami (50 %)</t>
+          <t>Nessim Mami (45 %)</t>
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>93431.89439165924</v>
+        <v>67156.67763721816</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>324271.1166930336</v>
+        <v>300858.8843351538</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>351942.194789947</v>
+        <v>264385.2219217446</v>
       </c>
       <c r="E6" s="13" t="n">
-        <v>535257.009421336</v>
+        <v>409099.1021651401</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>758051.3675243405</v>
+        <v>589344.5715329897</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>1008262.898254234</v>
+        <v>851545.8293109457</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>1283962.916601288</v>
+        <v>1177601.249548563</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>4355179.397675838</v>
+        <v>3659991.536451755</v>
       </c>
     </row>
     <row r="7">
@@ -2791,25 +2825,25 @@
         <v>0</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>28851.50554234641</v>
+        <v>4453.089984651087</v>
       </c>
       <c r="D7" s="11" t="n">
-        <v>175971.0973949735</v>
+        <v>146880.6788454136</v>
       </c>
       <c r="E7" s="11" t="n">
-        <v>267628.504710668</v>
+        <v>227277.2789806334</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>379025.6837621703</v>
+        <v>327413.6508516609</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>504131.4491271172</v>
+        <v>473081.0162838587</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>641981.4583006438</v>
+        <v>654222.9164158683</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>1997589.698837919</v>
+        <v>1833328.631362086</v>
       </c>
     </row>
     <row r="8">
@@ -2822,67 +2856,98 @@
         <v>0</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>28851.50554234641</v>
+        <v>4453.089984651087</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>175971.0973949735</v>
+        <v>146880.6788454136</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>267628.504710668</v>
+        <v>227277.2789806334</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>379025.6837621703</v>
+        <v>327413.6508516609</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>504131.4491271172</v>
+        <v>473081.0162838587</v>
       </c>
       <c r="H8" s="11" t="n">
-        <v>641981.4583006438</v>
+        <v>654222.9164158683</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>1997589.698837919</v>
+        <v>1833328.631362086</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Nazeh Ben Ammar (5 %)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>890.6179969302175</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>29376.13576908273</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>45455.45579612668</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>65482.73017033219</v>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>94616.20325677175</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>130844.5832831737</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>366665.7262724172</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>TOTAL distribué</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
-        <v>93431.89439165924</v>
-      </c>
-      <c r="C9" s="18" t="n">
-        <v>381974.1277777264</v>
-      </c>
-      <c r="D9" s="18" t="n">
-        <v>703884.3895798939</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>1070514.018842672</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>1516102.735048681</v>
-      </c>
-      <c r="G9" s="18" t="n">
-        <v>2016525.796508469</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>2567925.833202575</v>
-      </c>
-      <c r="I9" s="18" t="n">
-        <v>8350358.795351677</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>Nessim : capital remboursé fin An 2 · TRI ≈ 90 % · multiple 14.5× · total reçu 4,355,179 DT</t>
-        </is>
+      <c r="B10" s="18" t="n">
+        <v>67156.67763721816</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>310655.6823013861</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>587522.7153816546</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>909109.1159225334</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>1309654.603406644</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>1892324.065135435</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>2616891.665663473</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>7693314.525448345</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Nessim : capital remboursé fin An 2 · TRI ≈ 78 % · multiple 12.2× · total reçu 3,659,992 DT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Note : dividende déclaré au titre de l'exercice N, versé en N+1. 30 % du résultat conservé en réserve.</t>
         </is>

</xml_diff>